<commit_message>
Phase 2 Step A: author independent deal plans and batch truth oracle
</commit_message>
<xml_diff>
--- a/docs/RULEPACK_REVIEW.xlsx
+++ b/docs/RULEPACK_REVIEW.xlsx
@@ -4,9 +4,9 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="1-50-10-8" sheetId="1" r:id="rId1"/>
-    <sheet name="2-50-10-8-NF" sheetId="2" r:id="rId2"/>
+    <sheet name="2-50-10-8-SLA" sheetId="2" r:id="rId2"/>
     <sheet name="3-50-10-8-1" sheetId="3" r:id="rId3"/>
-    <sheet name="4-50-10-8-1-NF" sheetId="4" r:id="rId4"/>
+    <sheet name="4-50-10-8-1-SLA" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -3447,7 +3447,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B2" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C2" t="str">
         <v>ENT-01</v>
@@ -3491,7 +3491,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B3" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C3" t="str">
         <v>ENT-02</v>
@@ -3535,7 +3535,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B4" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C4" t="str">
         <v>ENT-03</v>
@@ -3579,7 +3579,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B5" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C5" t="str">
         <v>ENT-04</v>
@@ -3623,7 +3623,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B6" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C6" t="str">
         <v>ENT-05</v>
@@ -3667,7 +3667,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B7" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C7" t="str">
         <v>ENT-06</v>
@@ -3711,7 +3711,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B8" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C8" t="str">
         <v>ENT-07a</v>
@@ -3755,7 +3755,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B9" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C9" t="str">
         <v>ENT-07b</v>
@@ -3799,7 +3799,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B10" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C10" t="str">
         <v>GUA-01</v>
@@ -3843,7 +3843,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B11" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C11" t="str">
         <v>GUA-02</v>
@@ -3887,7 +3887,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B12" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C12" t="str">
         <v>GUA-03</v>
@@ -3931,7 +3931,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B13" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C13" t="str">
         <v>GUA-04</v>
@@ -3975,7 +3975,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B14" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C14" t="str">
         <v>GUA-05</v>
@@ -4019,7 +4019,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B15" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C15" t="str">
         <v>GUA-06</v>
@@ -4063,7 +4063,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B16" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C16" t="str">
         <v>GUA-07</v>
@@ -4107,7 +4107,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B17" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C17" t="str">
         <v>GUA-08a</v>
@@ -4151,7 +4151,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B18" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C18" t="str">
         <v>GUA-08b</v>
@@ -4195,7 +4195,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B19" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C19" t="str">
         <v>GUA-08c</v>
@@ -4239,7 +4239,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B20" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C20" t="str">
         <v>GUA-09a</v>
@@ -4283,7 +4283,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B21" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C21" t="str">
         <v>GUA-09b</v>
@@ -4327,7 +4327,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B22" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C22" t="str">
         <v>GUA-09c</v>
@@ -4371,7 +4371,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B23" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C23" t="str">
         <v>LND-01</v>
@@ -4415,7 +4415,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B24" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C24" t="str">
         <v>LND-02</v>
@@ -4459,7 +4459,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B25" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C25" t="str">
         <v>LND-03</v>
@@ -4503,7 +4503,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B26" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C26" t="str">
         <v>LND-04</v>
@@ -4547,7 +4547,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B27" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C27" t="str">
         <v>RE-01</v>
@@ -4591,7 +4591,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B28" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C28" t="str">
         <v>RE-02</v>
@@ -4635,7 +4635,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B29" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C29" t="str">
         <v>RE-03</v>
@@ -4679,7 +4679,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B30" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C30" t="str">
         <v>TGT-01</v>
@@ -4723,7 +4723,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B31" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C31" t="str">
         <v>TGT-02</v>
@@ -4767,7 +4767,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B32" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C32" t="str">
         <v>TGT-03</v>
@@ -4811,7 +4811,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B33" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C33" t="str">
         <v>TGT-04a</v>
@@ -4855,7 +4855,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B34" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C34" t="str">
         <v>TGT-04b</v>
@@ -4899,7 +4899,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B35" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C35" t="str">
         <v>TGT-05</v>
@@ -4943,7 +4943,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B36" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C36" t="str">
         <v>TGT-06</v>
@@ -4987,7 +4987,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B37" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C37" t="str">
         <v>TGT-07a</v>
@@ -5031,7 +5031,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B38" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C38" t="str">
         <v>TGT-07b</v>
@@ -5075,7 +5075,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B39" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C39" t="str">
         <v>TGT-08a</v>
@@ -5119,7 +5119,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B40" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C40" t="str">
         <v>TGT-08b</v>
@@ -5163,7 +5163,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B41" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C41" t="str">
         <v>TGT-09</v>
@@ -5207,7 +5207,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B42" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C42" t="str">
         <v>TGT-10a</v>
@@ -5251,7 +5251,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B43" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C43" t="str">
         <v>TGT-10b</v>
@@ -5295,7 +5295,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B44" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C44" t="str">
         <v>TGT-11</v>
@@ -5322,7 +5322,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K44" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Northfield synthetic lender addition: add-back support</v>
+        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: add-back support</v>
       </c>
       <c r="L44" t="str">
         <v/>
@@ -5339,7 +5339,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B45" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C45" t="str">
         <v>TGT-12a</v>
@@ -5383,7 +5383,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B46" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C46" t="str">
         <v>TGT-12b</v>
@@ -5427,7 +5427,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B47" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C47" t="str">
         <v>TGT-12c</v>
@@ -5471,7 +5471,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B48" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C48" t="str">
         <v>TXN-01</v>
@@ -5515,7 +5515,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B49" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C49" t="str">
         <v>TXN-02</v>
@@ -5559,7 +5559,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B50" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C50" t="str">
         <v>TXN-03</v>
@@ -5603,7 +5603,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B51" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C51" t="str">
         <v>TXN-04</v>
@@ -5647,7 +5647,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B52" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C52" t="str">
         <v>TXN-05</v>
@@ -5691,7 +5691,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B53" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C53" t="str">
         <v>TXN-06</v>
@@ -5735,7 +5735,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B54" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C54" t="str">
         <v>TXN-07</v>
@@ -5779,7 +5779,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B55" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C55" t="str">
         <v>TXN-08</v>
@@ -5823,7 +5823,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B56" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C56" t="str">
         <v>TXN-10a</v>
@@ -5850,7 +5850,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K56" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Northfield synthetic lender addition: non-compete</v>
+        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: non-compete</v>
       </c>
       <c r="L56" t="str">
         <v/>
@@ -5867,7 +5867,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B57" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C57" t="str">
         <v>TXN-10b</v>
@@ -5911,7 +5911,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B58" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C58" t="str">
         <v>TXN-10c</v>
@@ -5955,7 +5955,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B59" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C59" t="str">
         <v>CON-01</v>
@@ -5999,7 +5999,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B60" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C60" t="str">
         <v>CON-02</v>
@@ -6043,7 +6043,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B61" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C61" t="str">
         <v>CON-03</v>
@@ -6087,7 +6087,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B62" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C62" t="str">
         <v>CON-04</v>
@@ -6131,7 +6131,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B63" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C63" t="str">
         <v>CON-05</v>
@@ -6175,7 +6175,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B64" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C64" t="str">
         <v>CON-06</v>
@@ -6219,7 +6219,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B65" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C65" t="str">
         <v>CON-07</v>
@@ -6263,7 +6263,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B66" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C66" t="str">
         <v>CON-08</v>
@@ -6307,7 +6307,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B67" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C67" t="str">
         <v>CON-09</v>
@@ -6351,7 +6351,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B68" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C68" t="str">
         <v>CON-10</v>
@@ -6395,7 +6395,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B69" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C69" t="str">
         <v>CON-11</v>
@@ -6439,7 +6439,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B70" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C70" t="str">
         <v>CON-12</v>
@@ -6483,7 +6483,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B71" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C71" t="str">
         <v>CON-13</v>
@@ -6527,7 +6527,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B72" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C72" t="str">
         <v>CON-14</v>
@@ -6571,7 +6571,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B73" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C73" t="str">
         <v>CON-15</v>
@@ -6615,7 +6615,7 @@
         <v>sop-50-10-8</v>
       </c>
       <c r="B74" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C74" t="str">
         <v>CON-16</v>
@@ -9759,7 +9759,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B2" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C2" t="str">
         <v>ENT-01</v>
@@ -9803,7 +9803,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B3" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C3" t="str">
         <v>ENT-02</v>
@@ -9847,7 +9847,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B4" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C4" t="str">
         <v>ENT-03</v>
@@ -9891,7 +9891,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B5" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C5" t="str">
         <v>ENT-04</v>
@@ -9935,7 +9935,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B6" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C6" t="str">
         <v>ENT-05</v>
@@ -9979,7 +9979,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B7" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C7" t="str">
         <v>ENT-06</v>
@@ -10023,7 +10023,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B8" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C8" t="str">
         <v>ENT-07a</v>
@@ -10067,7 +10067,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B9" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C9" t="str">
         <v>ENT-07b</v>
@@ -10111,7 +10111,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B10" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C10" t="str">
         <v>GUA-01</v>
@@ -10155,7 +10155,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B11" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C11" t="str">
         <v>GUA-02</v>
@@ -10199,7 +10199,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B12" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C12" t="str">
         <v>GUA-03</v>
@@ -10243,7 +10243,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B13" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C13" t="str">
         <v>GUA-04</v>
@@ -10287,7 +10287,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B14" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C14" t="str">
         <v>GUA-05</v>
@@ -10331,7 +10331,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B15" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C15" t="str">
         <v>GUA-06</v>
@@ -10375,7 +10375,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B16" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C16" t="str">
         <v>GUA-07</v>
@@ -10419,7 +10419,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B17" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C17" t="str">
         <v>GUA-08a</v>
@@ -10463,7 +10463,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B18" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C18" t="str">
         <v>GUA-08b</v>
@@ -10507,7 +10507,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B19" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C19" t="str">
         <v>GUA-08c</v>
@@ -10551,7 +10551,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B20" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C20" t="str">
         <v>GUA-09a</v>
@@ -10595,7 +10595,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B21" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C21" t="str">
         <v>GUA-09b</v>
@@ -10639,7 +10639,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B22" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C22" t="str">
         <v>GUA-09c</v>
@@ -10683,7 +10683,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B23" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C23" t="str">
         <v>LND-01</v>
@@ -10727,7 +10727,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B24" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C24" t="str">
         <v>LND-02</v>
@@ -10771,7 +10771,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B25" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C25" t="str">
         <v>LND-03</v>
@@ -10815,7 +10815,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B26" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C26" t="str">
         <v>LND-04</v>
@@ -10859,7 +10859,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B27" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C27" t="str">
         <v>RE-01</v>
@@ -10903,7 +10903,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B28" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C28" t="str">
         <v>RE-02</v>
@@ -10947,7 +10947,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B29" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C29" t="str">
         <v>RE-03</v>
@@ -10991,7 +10991,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B30" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C30" t="str">
         <v>TGT-01</v>
@@ -11035,7 +11035,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B31" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C31" t="str">
         <v>TGT-02</v>
@@ -11079,7 +11079,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B32" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C32" t="str">
         <v>TGT-03</v>
@@ -11123,7 +11123,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B33" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C33" t="str">
         <v>TGT-04a</v>
@@ -11167,7 +11167,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B34" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C34" t="str">
         <v>TGT-04b</v>
@@ -11211,7 +11211,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B35" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C35" t="str">
         <v>TGT-05</v>
@@ -11255,7 +11255,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B36" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C36" t="str">
         <v>TGT-06</v>
@@ -11299,7 +11299,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B37" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C37" t="str">
         <v>TGT-07a</v>
@@ -11343,7 +11343,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B38" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C38" t="str">
         <v>TGT-07b</v>
@@ -11387,7 +11387,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B39" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C39" t="str">
         <v>TGT-08a</v>
@@ -11431,7 +11431,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B40" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C40" t="str">
         <v>TGT-08b</v>
@@ -11475,7 +11475,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B41" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C41" t="str">
         <v>TGT-09</v>
@@ -11519,7 +11519,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B42" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C42" t="str">
         <v>TGT-10a</v>
@@ -11563,7 +11563,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B43" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C43" t="str">
         <v>TGT-10b</v>
@@ -11607,7 +11607,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B44" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C44" t="str">
         <v>TGT-11</v>
@@ -11634,7 +11634,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K44" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Northfield synthetic lender addition: add-back support</v>
+        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: add-back support</v>
       </c>
       <c r="L44" t="str">
         <v/>
@@ -11651,7 +11651,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B45" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C45" t="str">
         <v>TGT-12a</v>
@@ -11695,7 +11695,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B46" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C46" t="str">
         <v>TGT-12b</v>
@@ -11739,7 +11739,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B47" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C47" t="str">
         <v>TGT-12c</v>
@@ -11783,7 +11783,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B48" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C48" t="str">
         <v>TXN-01</v>
@@ -11827,7 +11827,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B49" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C49" t="str">
         <v>TXN-02</v>
@@ -11871,7 +11871,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B50" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C50" t="str">
         <v>TXN-03</v>
@@ -11915,7 +11915,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B51" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C51" t="str">
         <v>TXN-04</v>
@@ -11959,7 +11959,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B52" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C52" t="str">
         <v>TXN-05</v>
@@ -12003,7 +12003,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B53" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C53" t="str">
         <v>TXN-06</v>
@@ -12047,7 +12047,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B54" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C54" t="str">
         <v>TXN-07</v>
@@ -12091,7 +12091,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B55" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C55" t="str">
         <v>TXN-08</v>
@@ -12135,7 +12135,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B56" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C56" t="str">
         <v>TXN-09</v>
@@ -12179,7 +12179,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B57" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C57" t="str">
         <v>TXN-10a</v>
@@ -12206,7 +12206,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K57" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Northfield synthetic lender addition: non-compete</v>
+        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: non-compete</v>
       </c>
       <c r="L57" t="str">
         <v/>
@@ -12223,7 +12223,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B58" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C58" t="str">
         <v>TXN-10b</v>
@@ -12267,7 +12267,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B59" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C59" t="str">
         <v>TXN-10c</v>
@@ -12311,7 +12311,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B60" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C60" t="str">
         <v>CON-01</v>
@@ -12355,7 +12355,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B61" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C61" t="str">
         <v>CON-02</v>
@@ -12399,7 +12399,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B62" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C62" t="str">
         <v>CON-03</v>
@@ -12443,7 +12443,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B63" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C63" t="str">
         <v>CON-04</v>
@@ -12487,7 +12487,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B64" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C64" t="str">
         <v>CON-05</v>
@@ -12531,7 +12531,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B65" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C65" t="str">
         <v>CON-06</v>
@@ -12575,7 +12575,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B66" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C66" t="str">
         <v>CON-07</v>
@@ -12619,7 +12619,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B67" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C67" t="str">
         <v>CON-08</v>
@@ -12663,7 +12663,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B68" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C68" t="str">
         <v>CON-09</v>
@@ -12707,7 +12707,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B69" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C69" t="str">
         <v>CON-10</v>
@@ -12751,7 +12751,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B70" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C70" t="str">
         <v>CON-11</v>
@@ -12795,7 +12795,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B71" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C71" t="str">
         <v>CON-12</v>
@@ -12839,7 +12839,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B72" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C72" t="str">
         <v>CON-13</v>
@@ -12883,7 +12883,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B73" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C73" t="str">
         <v>CON-14</v>
@@ -12927,7 +12927,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B74" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C74" t="str">
         <v>CON-15</v>
@@ -12971,7 +12971,7 @@
         <v>sop-50-10-8-1</v>
       </c>
       <c r="B75" t="str">
-        <v>northfield-bank</v>
+        <v>sample-lender-a</v>
       </c>
       <c r="C75" t="str">
         <v>CON-16</v>

</xml_diff>

<commit_message>
Rename product to LoanDocket
</commit_message>
<xml_diff>
--- a/docs/RULEPACK_REVIEW.xlsx
+++ b/docs/RULEPACK_REVIEW.xlsx
@@ -494,7 +494,7 @@
         <v>secondary</v>
       </c>
       <c r="K2" t="str">
-        <v>StatementsReady, How to Fill Out SBA Form 1919: revision 02/2025 and owner entries; the 100% ownership total and every-owner comparison are AcqFile seed conventions, stronger than the form’s minimum listing coverage.</v>
+        <v>StatementsReady, How to Fill Out SBA Form 1919: revision 02/2025 and owner entries; the 100% ownership total and every-owner comparison are LoanDocket seed conventions, stronger than the form’s minimum listing coverage.</v>
       </c>
       <c r="L2" t="str">
         <v>https://statementsready.com/blog/how-to-fill-out-sba-form-1919</v>
@@ -626,7 +626,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K5" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): EIN confirmation letter</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): EIN confirmation letter</v>
       </c>
       <c r="L5" t="str">
         <v/>
@@ -670,7 +670,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K6" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Buyer good standing; no inference from the secondary article citation to 13 CFR 120.420</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Buyer good standing; no inference from the secondary article citation to 13 CFR 120.420</v>
       </c>
       <c r="L6" t="str">
         <v/>
@@ -714,7 +714,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K7" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Includes indirect owners; manual facts permitted</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Includes indirect owners; manual facts permitted</v>
       </c>
       <c r="L7" t="str">
         <v/>
@@ -758,7 +758,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K8" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Business plan</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Business plan</v>
       </c>
       <c r="L8" t="str">
         <v/>
@@ -802,7 +802,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K9" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Projections with assumptions</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Projections with assumptions</v>
       </c>
       <c r="L9" t="str">
         <v/>
@@ -934,7 +934,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K12" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Resume or management profile</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Resume or management profile</v>
       </c>
       <c r="L12" t="str">
         <v/>
@@ -978,7 +978,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K13" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Government photo identification</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Government photo identification</v>
       </c>
       <c r="L13" t="str">
         <v/>
@@ -1022,7 +1022,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K14" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Evidence and manual lender discussion only; this is not a citizenship determination. Section A Ch.1 F differs between versions and later notices; see RULE_CANDIDATES.md.</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Evidence and manual lender discussion only; this is not a citizenship determination. Section A Ch.1 F differs between versions and later notices; see RULE_CANDIDATES.md.</v>
       </c>
       <c r="L14" t="str">
         <v/>
@@ -1110,7 +1110,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K16" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Two latest completed calendar months per declared cash source account; stronger than the cited 30-day evidence practice</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Two latest completed calendar months per declared cash source account; stronger than the cited 30-day evidence practice</v>
       </c>
       <c r="L16" t="str">
         <v/>
@@ -1418,7 +1418,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K23" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L23" t="str">
         <v/>
@@ -1462,7 +1462,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K24" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L24" t="str">
         <v/>
@@ -1506,7 +1506,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K25" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L25" t="str">
         <v/>
@@ -1550,7 +1550,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K26" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L26" t="str">
         <v/>
@@ -1594,7 +1594,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K27" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Real estate purchase contract</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Real estate purchase contract</v>
       </c>
       <c r="L27" t="str">
         <v/>
@@ -1638,7 +1638,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K28" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Real estate appraisal</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Real estate appraisal</v>
       </c>
       <c r="L28" t="str">
         <v/>
@@ -1682,7 +1682,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K29" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Environmental review</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Environmental review</v>
       </c>
       <c r="L29" t="str">
         <v/>
@@ -1858,7 +1858,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K33" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Receivables aging</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Receivables aging</v>
       </c>
       <c r="L33" t="str">
         <v/>
@@ -1902,7 +1902,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K34" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Payables aging</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Payables aging</v>
       </c>
       <c r="L34" t="str">
         <v/>
@@ -1990,7 +1990,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K36" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Signed 4506-C; 120-day signature window is a synthetic seed convention, not a claim about IRS validity</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Signed 4506-C; 120-day signature window is a synthetic seed convention, not a claim about IRS validity</v>
       </c>
       <c r="L36" t="str">
         <v/>
@@ -2078,7 +2078,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K38" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Lease assignment, consent or new terms</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Lease assignment, consent or new terms</v>
       </c>
       <c r="L38" t="str">
         <v/>
@@ -2122,7 +2122,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K39" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Equipment list</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Equipment list</v>
       </c>
       <c r="L39" t="str">
         <v/>
@@ -2166,7 +2166,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K40" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Inventory summary</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Inventory summary</v>
       </c>
       <c r="L40" t="str">
         <v/>
@@ -2210,7 +2210,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K41" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Operating licenses and permits</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Operating licenses and permits</v>
       </c>
       <c r="L41" t="str">
         <v/>
@@ -2298,7 +2298,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K43" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Franchise disclosure document</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Franchise disclosure document</v>
       </c>
       <c r="L43" t="str">
         <v/>
@@ -2342,7 +2342,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K44" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Signed letter of intent</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Signed letter of intent</v>
       </c>
       <c r="L44" t="str">
         <v/>
@@ -2430,7 +2430,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K46" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sources and uses</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Sources and uses</v>
       </c>
       <c r="L46" t="str">
         <v/>
@@ -2474,7 +2474,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K47" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Seller note or term sheet</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Seller note or term sheet</v>
       </c>
       <c r="L47" t="str">
         <v/>
@@ -2562,7 +2562,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K49" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Seller consulting or transition agreement</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Seller consulting or transition agreement</v>
       </c>
       <c r="L49" t="str">
         <v/>
@@ -2694,7 +2694,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K52" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L52" t="str">
         <v/>
@@ -2738,7 +2738,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K53" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L53" t="str">
         <v/>
@@ -2782,7 +2782,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K54" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L54" t="str">
         <v/>
@@ -2826,7 +2826,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K55" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L55" t="str">
         <v/>
@@ -2870,7 +2870,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K56" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L56" t="str">
         <v/>
@@ -2958,7 +2958,7 @@
         <v>sop</v>
       </c>
       <c r="K58" t="str">
-        <v>SOP 50 10 8, Section B Ch.1 C.2, Equity Requirements (C begins p.129); fixed 10% baseline is the AcqFile seed convention. Pagination is the section-start page in the official DOCX table of contents; see docs/RULE_SOURCES.md.</v>
+        <v>SOP 50 10 8, Section B Ch.1 C.2, Equity Requirements (C begins p.129); fixed 10% baseline is the LoanDocket seed convention. Pagination is the section-start page in the official DOCX table of contents; see docs/RULE_SOURCES.md.</v>
       </c>
       <c r="L58" t="str">
         <v>https://legacy.sba.gov/sites/default/files/2025-05/SOP%2050%2010%208%20Technical%20Updates%20effective%206.1.2025.docx</v>
@@ -3002,7 +3002,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K59" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L59" t="str">
         <v/>
@@ -3046,7 +3046,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K60" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L60" t="str">
         <v/>
@@ -3090,7 +3090,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K61" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L61" t="str">
         <v/>
@@ -3134,7 +3134,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K62" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L62" t="str">
         <v/>
@@ -3178,7 +3178,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K63" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L63" t="str">
         <v/>
@@ -3222,7 +3222,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K64" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Ten-year review horizon; not a universal lease term determination</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Ten-year review horizon; not a universal lease term determination</v>
       </c>
       <c r="L64" t="str">
         <v/>
@@ -3310,7 +3310,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K66" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L66" t="str">
         <v/>
@@ -3354,7 +3354,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K67" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L67" t="str">
         <v/>
@@ -3474,7 +3474,7 @@
         <v>secondary</v>
       </c>
       <c r="K2" t="str">
-        <v>StatementsReady, How to Fill Out SBA Form 1919: revision 02/2025 and owner entries; the 100% ownership total and every-owner comparison are AcqFile seed conventions, stronger than the form’s minimum listing coverage.</v>
+        <v>StatementsReady, How to Fill Out SBA Form 1919: revision 02/2025 and owner entries; the 100% ownership total and every-owner comparison are LoanDocket seed conventions, stronger than the form’s minimum listing coverage.</v>
       </c>
       <c r="L2" t="str">
         <v>https://statementsready.com/blog/how-to-fill-out-sba-form-1919</v>
@@ -3606,7 +3606,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K5" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): EIN confirmation letter</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): EIN confirmation letter</v>
       </c>
       <c r="L5" t="str">
         <v/>
@@ -3650,7 +3650,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K6" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Buyer good standing; no inference from the secondary article citation to 13 CFR 120.420</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Buyer good standing; no inference from the secondary article citation to 13 CFR 120.420</v>
       </c>
       <c r="L6" t="str">
         <v/>
@@ -3694,7 +3694,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K7" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Includes indirect owners; manual facts permitted</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Includes indirect owners; manual facts permitted</v>
       </c>
       <c r="L7" t="str">
         <v/>
@@ -3738,7 +3738,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K8" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Business plan</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Business plan</v>
       </c>
       <c r="L8" t="str">
         <v/>
@@ -3782,7 +3782,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K9" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Projections with assumptions</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Projections with assumptions</v>
       </c>
       <c r="L9" t="str">
         <v/>
@@ -3914,7 +3914,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K12" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Resume or management profile</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Resume or management profile</v>
       </c>
       <c r="L12" t="str">
         <v/>
@@ -3958,7 +3958,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K13" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Government photo identification</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Government photo identification</v>
       </c>
       <c r="L13" t="str">
         <v/>
@@ -4002,7 +4002,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K14" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Evidence and manual lender discussion only; this is not a citizenship determination. Section A Ch.1 F differs between versions and later notices; see RULE_CANDIDATES.md.</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Evidence and manual lender discussion only; this is not a citizenship determination. Section A Ch.1 F differs between versions and later notices; see RULE_CANDIDATES.md.</v>
       </c>
       <c r="L14" t="str">
         <v/>
@@ -4090,7 +4090,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K16" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Two latest completed calendar months per declared cash source account; stronger than the cited 30-day evidence practice</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Two latest completed calendar months per declared cash source account; stronger than the cited 30-day evidence practice</v>
       </c>
       <c r="L16" t="str">
         <v/>
@@ -4398,7 +4398,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K23" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L23" t="str">
         <v/>
@@ -4442,7 +4442,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K24" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L24" t="str">
         <v/>
@@ -4486,7 +4486,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K25" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L25" t="str">
         <v/>
@@ -4530,7 +4530,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K26" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L26" t="str">
         <v/>
@@ -4574,7 +4574,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K27" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Real estate purchase contract</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Real estate purchase contract</v>
       </c>
       <c r="L27" t="str">
         <v/>
@@ -4618,7 +4618,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K28" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Real estate appraisal</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Real estate appraisal</v>
       </c>
       <c r="L28" t="str">
         <v/>
@@ -4662,7 +4662,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K29" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Environmental review</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Environmental review</v>
       </c>
       <c r="L29" t="str">
         <v/>
@@ -4838,7 +4838,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K33" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Receivables aging</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Receivables aging</v>
       </c>
       <c r="L33" t="str">
         <v/>
@@ -4882,7 +4882,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K34" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Payables aging</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Payables aging</v>
       </c>
       <c r="L34" t="str">
         <v/>
@@ -4970,7 +4970,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K36" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Signed 4506-C; 120-day signature window is a synthetic seed convention, not a claim about IRS validity</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Signed 4506-C; 120-day signature window is a synthetic seed convention, not a claim about IRS validity</v>
       </c>
       <c r="L36" t="str">
         <v/>
@@ -5058,7 +5058,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K38" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Lease assignment, consent or new terms</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Lease assignment, consent or new terms</v>
       </c>
       <c r="L38" t="str">
         <v/>
@@ -5102,7 +5102,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K39" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Equipment list</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Equipment list</v>
       </c>
       <c r="L39" t="str">
         <v/>
@@ -5146,7 +5146,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K40" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Inventory summary</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Inventory summary</v>
       </c>
       <c r="L40" t="str">
         <v/>
@@ -5190,7 +5190,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K41" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Operating licenses and permits</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Operating licenses and permits</v>
       </c>
       <c r="L41" t="str">
         <v/>
@@ -5278,7 +5278,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K43" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Franchise disclosure document</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Franchise disclosure document</v>
       </c>
       <c r="L43" t="str">
         <v/>
@@ -5322,7 +5322,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K44" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: add-back support</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: add-back support</v>
       </c>
       <c r="L44" t="str">
         <v/>
@@ -5366,7 +5366,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K45" t="str">
-        <v>AcqFile SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
+        <v>LoanDocket SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
       </c>
       <c r="L45" t="str">
         <v/>
@@ -5410,7 +5410,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K46" t="str">
-        <v>AcqFile SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
+        <v>LoanDocket SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
       </c>
       <c r="L46" t="str">
         <v/>
@@ -5454,7 +5454,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K47" t="str">
-        <v>AcqFile SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
+        <v>LoanDocket SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
       </c>
       <c r="L47" t="str">
         <v/>
@@ -5498,7 +5498,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K48" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Signed letter of intent</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Signed letter of intent</v>
       </c>
       <c r="L48" t="str">
         <v/>
@@ -5586,7 +5586,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K50" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sources and uses</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Sources and uses</v>
       </c>
       <c r="L50" t="str">
         <v/>
@@ -5630,7 +5630,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K51" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Seller note or term sheet</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Seller note or term sheet</v>
       </c>
       <c r="L51" t="str">
         <v/>
@@ -5718,7 +5718,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K53" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Seller consulting or transition agreement</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Seller consulting or transition agreement</v>
       </c>
       <c r="L53" t="str">
         <v/>
@@ -5850,7 +5850,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K56" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: non-compete</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: non-compete</v>
       </c>
       <c r="L56" t="str">
         <v/>
@@ -5894,7 +5894,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K57" t="str">
-        <v>AcqFile SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
+        <v>LoanDocket SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
       </c>
       <c r="L57" t="str">
         <v/>
@@ -5938,7 +5938,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K58" t="str">
-        <v>AcqFile SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
+        <v>LoanDocket SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
       </c>
       <c r="L58" t="str">
         <v/>
@@ -5982,7 +5982,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K59" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L59" t="str">
         <v/>
@@ -6026,7 +6026,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K60" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L60" t="str">
         <v/>
@@ -6070,7 +6070,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K61" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L61" t="str">
         <v/>
@@ -6114,7 +6114,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K62" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L62" t="str">
         <v/>
@@ -6158,7 +6158,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K63" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L63" t="str">
         <v/>
@@ -6246,7 +6246,7 @@
         <v>sop</v>
       </c>
       <c r="K65" t="str">
-        <v>SOP 50 10 8, Section B Ch.1 C.2, Equity Requirements (C begins p.129); fixed 10% baseline is the AcqFile seed convention. Pagination is the section-start page in the official DOCX table of contents; see docs/RULE_SOURCES.md.</v>
+        <v>SOP 50 10 8, Section B Ch.1 C.2, Equity Requirements (C begins p.129); fixed 10% baseline is the LoanDocket seed convention. Pagination is the section-start page in the official DOCX table of contents; see docs/RULE_SOURCES.md.</v>
       </c>
       <c r="L65" t="str">
         <v>https://legacy.sba.gov/sites/default/files/2025-05/SOP%2050%2010%208%20Technical%20Updates%20effective%206.1.2025.docx</v>
@@ -6290,7 +6290,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K66" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L66" t="str">
         <v/>
@@ -6334,7 +6334,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K67" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L67" t="str">
         <v/>
@@ -6378,7 +6378,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K68" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L68" t="str">
         <v/>
@@ -6422,7 +6422,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K69" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L69" t="str">
         <v/>
@@ -6466,7 +6466,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K70" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L70" t="str">
         <v/>
@@ -6510,7 +6510,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K71" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Ten-year review horizon; not a universal lease term determination</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Ten-year review horizon; not a universal lease term determination</v>
       </c>
       <c r="L71" t="str">
         <v/>
@@ -6598,7 +6598,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K73" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L73" t="str">
         <v/>
@@ -6642,7 +6642,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K74" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L74" t="str">
         <v/>
@@ -6762,7 +6762,7 @@
         <v>secondary</v>
       </c>
       <c r="K2" t="str">
-        <v>StatementsReady, How to Fill Out SBA Form 1919: revision 02/2025 and owner entries; the 100% ownership total and every-owner comparison are AcqFile seed conventions, stronger than the form’s minimum listing coverage.</v>
+        <v>StatementsReady, How to Fill Out SBA Form 1919: revision 02/2025 and owner entries; the 100% ownership total and every-owner comparison are LoanDocket seed conventions, stronger than the form’s minimum listing coverage.</v>
       </c>
       <c r="L2" t="str">
         <v>https://statementsready.com/blog/how-to-fill-out-sba-form-1919</v>
@@ -6894,7 +6894,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K5" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): EIN confirmation letter</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): EIN confirmation letter</v>
       </c>
       <c r="L5" t="str">
         <v/>
@@ -6938,7 +6938,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K6" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Buyer good standing; no inference from the secondary article citation to 13 CFR 120.420</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Buyer good standing; no inference from the secondary article citation to 13 CFR 120.420</v>
       </c>
       <c r="L6" t="str">
         <v/>
@@ -6982,7 +6982,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K7" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Includes indirect owners; manual facts permitted</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Includes indirect owners; manual facts permitted</v>
       </c>
       <c r="L7" t="str">
         <v/>
@@ -7026,7 +7026,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K8" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Business plan</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Business plan</v>
       </c>
       <c r="L8" t="str">
         <v/>
@@ -7070,7 +7070,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K9" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Projections with assumptions</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Projections with assumptions</v>
       </c>
       <c r="L9" t="str">
         <v/>
@@ -7202,7 +7202,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K12" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Resume or management profile</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Resume or management profile</v>
       </c>
       <c r="L12" t="str">
         <v/>
@@ -7246,7 +7246,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K13" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Government photo identification</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Government photo identification</v>
       </c>
       <c r="L13" t="str">
         <v/>
@@ -7290,7 +7290,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K14" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Evidence and manual lender discussion only; this is not a citizenship determination. Section A Ch.1 F differs between versions and later notices; see RULE_CANDIDATES.md.</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Evidence and manual lender discussion only; this is not a citizenship determination. Section A Ch.1 F differs between versions and later notices; see RULE_CANDIDATES.md.</v>
       </c>
       <c r="L14" t="str">
         <v/>
@@ -7378,7 +7378,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K16" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Two latest completed calendar months per declared cash source account; stronger than the cited 30-day evidence practice</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Two latest completed calendar months per declared cash source account; stronger than the cited 30-day evidence practice</v>
       </c>
       <c r="L16" t="str">
         <v/>
@@ -7686,7 +7686,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K23" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L23" t="str">
         <v/>
@@ -7730,7 +7730,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K24" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L24" t="str">
         <v/>
@@ -7774,7 +7774,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K25" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L25" t="str">
         <v/>
@@ -7818,7 +7818,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K26" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L26" t="str">
         <v/>
@@ -7862,7 +7862,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K27" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Real estate purchase contract</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Real estate purchase contract</v>
       </c>
       <c r="L27" t="str">
         <v/>
@@ -7906,7 +7906,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K28" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Real estate appraisal</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Real estate appraisal</v>
       </c>
       <c r="L28" t="str">
         <v/>
@@ -7950,7 +7950,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K29" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Environmental review</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Environmental review</v>
       </c>
       <c r="L29" t="str">
         <v/>
@@ -8126,7 +8126,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K33" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Receivables aging</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Receivables aging</v>
       </c>
       <c r="L33" t="str">
         <v/>
@@ -8170,7 +8170,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K34" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Payables aging</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Payables aging</v>
       </c>
       <c r="L34" t="str">
         <v/>
@@ -8258,7 +8258,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K36" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Signed 4506-C; 120-day signature window is a synthetic seed convention, not a claim about IRS validity</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Signed 4506-C; 120-day signature window is a synthetic seed convention, not a claim about IRS validity</v>
       </c>
       <c r="L36" t="str">
         <v/>
@@ -8346,7 +8346,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K38" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Lease assignment, consent or new terms</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Lease assignment, consent or new terms</v>
       </c>
       <c r="L38" t="str">
         <v/>
@@ -8390,7 +8390,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K39" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Equipment list</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Equipment list</v>
       </c>
       <c r="L39" t="str">
         <v/>
@@ -8434,7 +8434,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K40" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Inventory summary</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Inventory summary</v>
       </c>
       <c r="L40" t="str">
         <v/>
@@ -8478,7 +8478,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K41" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Operating licenses and permits</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Operating licenses and permits</v>
       </c>
       <c r="L41" t="str">
         <v/>
@@ -8566,7 +8566,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K43" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Franchise disclosure document</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Franchise disclosure document</v>
       </c>
       <c r="L43" t="str">
         <v/>
@@ -8610,7 +8610,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K44" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Signed letter of intent</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Signed letter of intent</v>
       </c>
       <c r="L44" t="str">
         <v/>
@@ -8698,7 +8698,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K46" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sources and uses</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Sources and uses</v>
       </c>
       <c r="L46" t="str">
         <v/>
@@ -8742,7 +8742,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K47" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Seller note or term sheet</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Seller note or term sheet</v>
       </c>
       <c r="L47" t="str">
         <v/>
@@ -8830,7 +8830,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K49" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Seller consulting or transition agreement</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Seller consulting or transition agreement</v>
       </c>
       <c r="L49" t="str">
         <v/>
@@ -9006,7 +9006,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K53" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L53" t="str">
         <v/>
@@ -9050,7 +9050,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K54" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L54" t="str">
         <v/>
@@ -9094,7 +9094,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K55" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L55" t="str">
         <v/>
@@ -9138,7 +9138,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K56" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L56" t="str">
         <v/>
@@ -9182,7 +9182,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K57" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L57" t="str">
         <v/>
@@ -9270,7 +9270,7 @@
         <v>sop</v>
       </c>
       <c r="K59" t="str">
-        <v>SOP 50 10 8.1, Appendix 15 C, Limited Equity Injection Sources (C begins p.350); fixed 10% baseline is the AcqFile seed convention. Pagination is the section-start page in the official DOCX table of contents; see docs/RULE_SOURCES.md.</v>
+        <v>SOP 50 10 8.1, Appendix 15 C, Limited Equity Injection Sources (C begins p.350); fixed 10% baseline is the LoanDocket seed convention. Pagination is the section-start page in the official DOCX table of contents; see docs/RULE_SOURCES.md.</v>
       </c>
       <c r="L59" t="str">
         <v>https://legacy.sba.gov/sites/default/files/2026-08/SOP%2050%2010%208.1%20effective%2010.1.2026_0.docx</v>
@@ -9314,7 +9314,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K60" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L60" t="str">
         <v/>
@@ -9358,7 +9358,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K61" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L61" t="str">
         <v/>
@@ -9402,7 +9402,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K62" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L62" t="str">
         <v/>
@@ -9446,7 +9446,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K63" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L63" t="str">
         <v/>
@@ -9490,7 +9490,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K64" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L64" t="str">
         <v/>
@@ -9534,7 +9534,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K65" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Ten-year review horizon; not a universal lease term determination</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Ten-year review horizon; not a universal lease term determination</v>
       </c>
       <c r="L65" t="str">
         <v/>
@@ -9622,7 +9622,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K67" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L67" t="str">
         <v/>
@@ -9666,7 +9666,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K68" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L68" t="str">
         <v/>
@@ -9786,7 +9786,7 @@
         <v>secondary</v>
       </c>
       <c r="K2" t="str">
-        <v>StatementsReady, How to Fill Out SBA Form 1919: revision 02/2025 and owner entries; the 100% ownership total and every-owner comparison are AcqFile seed conventions, stronger than the form’s minimum listing coverage.</v>
+        <v>StatementsReady, How to Fill Out SBA Form 1919: revision 02/2025 and owner entries; the 100% ownership total and every-owner comparison are LoanDocket seed conventions, stronger than the form’s minimum listing coverage.</v>
       </c>
       <c r="L2" t="str">
         <v>https://statementsready.com/blog/how-to-fill-out-sba-form-1919</v>
@@ -9918,7 +9918,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K5" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): EIN confirmation letter</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): EIN confirmation letter</v>
       </c>
       <c r="L5" t="str">
         <v/>
@@ -9962,7 +9962,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K6" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Buyer good standing; no inference from the secondary article citation to 13 CFR 120.420</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Buyer good standing; no inference from the secondary article citation to 13 CFR 120.420</v>
       </c>
       <c r="L6" t="str">
         <v/>
@@ -10006,7 +10006,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K7" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Includes indirect owners; manual facts permitted</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Includes indirect owners; manual facts permitted</v>
       </c>
       <c r="L7" t="str">
         <v/>
@@ -10050,7 +10050,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K8" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Business plan</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Business plan</v>
       </c>
       <c r="L8" t="str">
         <v/>
@@ -10094,7 +10094,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K9" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Projections with assumptions</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Projections with assumptions</v>
       </c>
       <c r="L9" t="str">
         <v/>
@@ -10226,7 +10226,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K12" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Resume or management profile</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Resume or management profile</v>
       </c>
       <c r="L12" t="str">
         <v/>
@@ -10270,7 +10270,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K13" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Government photo identification</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Government photo identification</v>
       </c>
       <c r="L13" t="str">
         <v/>
@@ -10314,7 +10314,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K14" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Evidence and manual lender discussion only; this is not a citizenship determination. Section A Ch.1 F differs between versions and later notices; see RULE_CANDIDATES.md.</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Evidence and manual lender discussion only; this is not a citizenship determination. Section A Ch.1 F differs between versions and later notices; see RULE_CANDIDATES.md.</v>
       </c>
       <c r="L14" t="str">
         <v/>
@@ -10402,7 +10402,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K16" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Two latest completed calendar months per declared cash source account; stronger than the cited 30-day evidence practice</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Two latest completed calendar months per declared cash source account; stronger than the cited 30-day evidence practice</v>
       </c>
       <c r="L16" t="str">
         <v/>
@@ -10710,7 +10710,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K23" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L23" t="str">
         <v/>
@@ -10754,7 +10754,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K24" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L24" t="str">
         <v/>
@@ -10798,7 +10798,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K25" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L25" t="str">
         <v/>
@@ -10842,7 +10842,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K26" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Always-visible lender work tracking; no borrower evidence requested</v>
       </c>
       <c r="L26" t="str">
         <v/>
@@ -10886,7 +10886,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K27" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Real estate purchase contract</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Real estate purchase contract</v>
       </c>
       <c r="L27" t="str">
         <v/>
@@ -10930,7 +10930,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K28" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Real estate appraisal</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Real estate appraisal</v>
       </c>
       <c r="L28" t="str">
         <v/>
@@ -10974,7 +10974,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K29" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Environmental review</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Environmental review</v>
       </c>
       <c r="L29" t="str">
         <v/>
@@ -11150,7 +11150,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K33" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Receivables aging</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Receivables aging</v>
       </c>
       <c r="L33" t="str">
         <v/>
@@ -11194,7 +11194,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K34" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Payables aging</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Payables aging</v>
       </c>
       <c r="L34" t="str">
         <v/>
@@ -11282,7 +11282,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K36" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Signed 4506-C; 120-day signature window is a synthetic seed convention, not a claim about IRS validity</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Signed 4506-C; 120-day signature window is a synthetic seed convention, not a claim about IRS validity</v>
       </c>
       <c r="L36" t="str">
         <v/>
@@ -11370,7 +11370,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K38" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Lease assignment, consent or new terms</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Lease assignment, consent or new terms</v>
       </c>
       <c r="L38" t="str">
         <v/>
@@ -11414,7 +11414,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K39" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Equipment list</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Equipment list</v>
       </c>
       <c r="L39" t="str">
         <v/>
@@ -11458,7 +11458,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K40" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Inventory summary</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Inventory summary</v>
       </c>
       <c r="L40" t="str">
         <v/>
@@ -11502,7 +11502,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K41" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Operating licenses and permits</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Operating licenses and permits</v>
       </c>
       <c r="L41" t="str">
         <v/>
@@ -11590,7 +11590,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K43" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Franchise disclosure document</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Franchise disclosure document</v>
       </c>
       <c r="L43" t="str">
         <v/>
@@ -11634,7 +11634,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K44" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: add-back support</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: add-back support</v>
       </c>
       <c r="L44" t="str">
         <v/>
@@ -11678,7 +11678,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K45" t="str">
-        <v>AcqFile SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
+        <v>LoanDocket SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
       </c>
       <c r="L45" t="str">
         <v/>
@@ -11722,7 +11722,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K46" t="str">
-        <v>AcqFile SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
+        <v>LoanDocket SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
       </c>
       <c r="L46" t="str">
         <v/>
@@ -11766,7 +11766,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K47" t="str">
-        <v>AcqFile SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
+        <v>LoanDocket SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
       </c>
       <c r="L47" t="str">
         <v/>
@@ -11810,7 +11810,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K48" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Signed letter of intent</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Signed letter of intent</v>
       </c>
       <c r="L48" t="str">
         <v/>
@@ -11898,7 +11898,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K50" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sources and uses</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Sources and uses</v>
       </c>
       <c r="L50" t="str">
         <v/>
@@ -11942,7 +11942,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K51" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Seller note or term sheet</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Seller note or term sheet</v>
       </c>
       <c r="L51" t="str">
         <v/>
@@ -12030,7 +12030,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K53" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Seller consulting or transition agreement</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Seller consulting or transition agreement</v>
       </c>
       <c r="L53" t="str">
         <v/>
@@ -12206,7 +12206,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K57" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: non-compete</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Sample Lender A synthetic lender addition: non-compete</v>
       </c>
       <c r="L57" t="str">
         <v/>
@@ -12250,7 +12250,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K58" t="str">
-        <v>AcqFile SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
+        <v>LoanDocket SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
       </c>
       <c r="L58" t="str">
         <v/>
@@ -12294,7 +12294,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K59" t="str">
-        <v>AcqFile SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
+        <v>LoanDocket SPEC Section 13 optional overlay seed; inactive unless a lender configuration explicitly requires it.</v>
       </c>
       <c r="L59" t="str">
         <v/>
@@ -12338,7 +12338,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K60" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L60" t="str">
         <v/>
@@ -12382,7 +12382,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K61" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L61" t="str">
         <v/>
@@ -12426,7 +12426,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K62" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L62" t="str">
         <v/>
@@ -12470,7 +12470,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K63" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L63" t="str">
         <v/>
@@ -12514,7 +12514,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K64" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L64" t="str">
         <v/>
@@ -12602,7 +12602,7 @@
         <v>sop</v>
       </c>
       <c r="K66" t="str">
-        <v>SOP 50 10 8.1, Appendix 15 C, Limited Equity Injection Sources (C begins p.350); fixed 10% baseline is the AcqFile seed convention. Pagination is the section-start page in the official DOCX table of contents; see docs/RULE_SOURCES.md.</v>
+        <v>SOP 50 10 8.1, Appendix 15 C, Limited Equity Injection Sources (C begins p.350); fixed 10% baseline is the LoanDocket seed convention. Pagination is the section-start page in the official DOCX table of contents; see docs/RULE_SOURCES.md.</v>
       </c>
       <c r="L66" t="str">
         <v>https://legacy.sba.gov/sites/default/files/2026-08/SOP%2050%2010%208.1%20effective%2010.1.2026_0.docx</v>
@@ -12646,7 +12646,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K67" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L67" t="str">
         <v/>
@@ -12690,7 +12690,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K68" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L68" t="str">
         <v/>
@@ -12734,7 +12734,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K69" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L69" t="str">
         <v/>
@@ -12778,7 +12778,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K70" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L70" t="str">
         <v/>
@@ -12822,7 +12822,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K71" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L71" t="str">
         <v/>
@@ -12866,7 +12866,7 @@
         <v>lender_convention</v>
       </c>
       <c r="K72" t="str">
-        <v>AcqFile synthetic seed convention (SPEC Section 13; unverified): Ten-year review horizon; not a universal lease term determination</v>
+        <v>LoanDocket synthetic seed convention (SPEC Section 13; unverified): Ten-year review horizon; not a universal lease term determination</v>
       </c>
       <c r="L72" t="str">
         <v/>
@@ -12954,7 +12954,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K74" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L74" t="str">
         <v/>
@@ -12998,7 +12998,7 @@
         <v>internal_consistency</v>
       </c>
       <c r="K75" t="str">
-        <v>AcqFile SPEC Section 13: internal consistency comparison; no lending determination.</v>
+        <v>LoanDocket SPEC Section 13: internal consistency comparison; no lending determination.</v>
       </c>
       <c r="L75" t="str">
         <v/>

</xml_diff>